<commit_message>
Tighten profit briefing conclusions for leadership review
Rewrite the summary page into one sentence, four short conclusions,
and four decision items; keep weekly detail as an appendix table.

Co-authored-by: ghg131419-cloud <ghg131419-cloud@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/天猫近3月数据_分析结果/天猫利润分析.xlsx
+++ b/天猫近3月数据_分析结果/天猫利润分析.xlsx
@@ -29,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +64,21 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -93,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -115,11 +130,12 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,6 +176,29 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,7 +565,621 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>天猫利润分析 · 领导一页纸</t>
+        </is>
+      </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
+      <c r="D1" s="19" t="n"/>
+      <c r="E1" s="19" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>口径：ID周损益｜推广后净利润｜5.11–8.2</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="n"/>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
+      <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>一句话</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>亏在大链接：量掉的时候利润掉，量回来时又被推广费吃掉；大大包不是主因。</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>核心结论</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>结论</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>结论1</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>近三个月一直在亏；最好一周是7.6（约-4100），之后又往下掉。</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>结论2</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>这波回落不是大大包的问题，主责在大链接：先是袋面主链销量掉，后是袋面次链推广加太猛。</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>结论3</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>结构上，袋面主/次链 + 杯面主链长期贡献大部分亏损；巴东新链接也在持续失血。</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>结论4</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>要抓三件事：控主链投产、砍低效推广、巴东减投验证；大大包只控推广侵蚀即可。</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>请拍板</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>① 立刻复盘袋面主链接：成交为何掉、推广前利润为何掉。</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>② 压降袋面次链接、30包等低效花费，先把费率打下来。</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>③ 巴东链接减投/停投一周看结果。</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>④ 大大包保留自然利润，严控加投。</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>附表：ID周合计（备查）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>周次</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>成交金额</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>推广前利润</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>推广花费</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>环比_推广后</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>环比_推广前</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>环比_推广费</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>推广费率</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>下降主因</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>5.11-5.17</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>118254.3200000011</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>15585.09100000004</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>22199.84999999998</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>-6308.342962264105</v>
+      </c>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="12" t="n">
+        <v>0.1877297167663708</v>
+      </c>
+      <c r="J22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>5.25-5.31</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>123376.8700000012</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>16530.79100000003</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>22867.12</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>-6519.925981132038</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>-211.5830188679329</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>945.6999999999898</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>667.270000000015</v>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v>0.1853436547709451</v>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>主要是推广费上升</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>6.15-6.21</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>102107.7300000007</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>13774.47300000003</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>19489.66</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>-6627.168509433931</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>-107.2425283018929</v>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>-2756.317999999999</v>
+      </c>
+      <c r="H24" s="11" t="n">
+        <v>-3377.460000000003</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>0.1908735019376091</v>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>主要是推广前利润下降</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>6.22-6.28</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>86704.38000000019</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>11721.55400000001</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>17051.12</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>-6338.785622641502</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>288.3828867924285</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <v>-2052.91900000002</v>
+      </c>
+      <c r="H25" s="11" t="n">
+        <v>-2438.539999999997</v>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v>0.1966581157722362</v>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>本期改善</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>6.29-7.5</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>93257.14000000031</v>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>12985.26300000003</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>17356.51</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>-5229.755867924498</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>1109.029754717005</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>1263.709000000019</v>
+      </c>
+      <c r="H26" s="10" t="n">
+        <v>305.3899999999994</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>0.186114543079489</v>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>本期改善</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>7.6-7.12</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>120624.1200000009</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>16853.98700000001</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>20166.80900000001</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>-4108.993188679236</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>1120.762679245261</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>3868.723999999982</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>2810.299000000014</v>
+      </c>
+      <c r="I27" s="15" t="n">
+        <v>0.1671872010340872</v>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>本期改善</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>7.13-7.19</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>100698.0300000007</v>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>13663.37600000004</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>17570.48999999999</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>-5181.567396226362</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>-1072.574207547125</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>-3190.610999999972</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>-2596.319000000025</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>0.1744869288902659</v>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>主要是推广前利润下降</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>7.20-7.26</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>98448.25000000061</v>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>13513.29000000004</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>18177.49</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>-5613.776037735816</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>-432.2086415094545</v>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>-150.0859999999975</v>
+      </c>
+      <c r="H29" s="10" t="n">
+        <v>607.0000000000146</v>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v>0.1846400520070178</v>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>主要是推广费上升</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>7.27-8.2</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>107467.6600000008</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>15014.01200000004</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>19204.37726581657</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>-5109.368381499395</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>504.4076562364216</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>1500.722</v>
+      </c>
+      <c r="H30" s="10" t="n">
+        <v>1026.887265816571</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>0.1786991292619233</v>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>本期改善</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -543,552 +1196,6 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>天猫近3个月利润分析 · 干净汇报版</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>主口径：ID周损益 · 净利润(推广后)｜周次：5.11–8.2（9个已校验单周）｜单位：元</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>店铺周报仅作附录对照，不与ID成交金额直接混比</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>一、核心结论</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>内容</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>结论1</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>最好周为 7.6-7.12（推广后 -4,109）。之后两周回落：7.13 -5,182（-1,073），7.20 -5,614（-432）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>结论2</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>7.6→7.13 主因是推广前利润下降（随成交回落）。拖累TOP3：668566625747 袋面主链接（-666）、649369494424 24包经典/牛系列（-211）、648600900806 30包（-202）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>结论3</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>7.13→7.20 更突出推广费上升。恶化最大：649361890551 袋面次链接（推广后 -259，推广费 +529）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>结论4</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>每周绝对亏损长期集中在袋面次链接、袋面主链接、杯面主链接；巴东牛肉等新链接持续大额亏损。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>结论5</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>原味大大包：推广前有利润，但推广后净贡献弱，不是近周回落第一责任。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>结论6</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>5.11→7.27 整段：成交 118,254→107,468（-9.1%），推广后 -6,308→-5,109（亏损略收窄）。不是“整段量增利降”。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>二、建议</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>1. 优先复盘袋面主链接成交与推广前利润下滑（阶段一）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>2. 压降袋面次链接、30包等低效推广（阶段二）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>3. 巴东牛肉单独评估减投/停投。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>4. 大大包保留推广前利润，严控推广侵蚀。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>三、ID周合计趋势（主表）</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>周次</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>成交金额</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>推广前利润</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>推广花费</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>推广后利润</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>环比_推广后</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>环比_推广前</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>环比_推广费</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>推广费率</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>下降主因</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>5.11-5.17</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>118254.3200000011</v>
-      </c>
-      <c r="C22" s="10" t="n">
-        <v>15585.09100000004</v>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>22199.84999999998</v>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>-6308.342962264105</v>
-      </c>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="8" t="n"/>
-      <c r="I22" s="12" t="n">
-        <v>0.1877297167663708</v>
-      </c>
-      <c r="J22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>5.25-5.31</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n">
-        <v>123376.8700000012</v>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>16530.79100000003</v>
-      </c>
-      <c r="D23" s="14" t="n">
-        <v>22867.12</v>
-      </c>
-      <c r="E23" s="11" t="n">
-        <v>-6519.925981132038</v>
-      </c>
-      <c r="F23" s="11" t="n">
-        <v>-211.5830188679329</v>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>945.6999999999898</v>
-      </c>
-      <c r="H23" s="10" t="n">
-        <v>667.270000000015</v>
-      </c>
-      <c r="I23" s="15" t="n">
-        <v>0.1853436547709451</v>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>主要是推广费上升</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>6.15-6.21</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="n">
-        <v>102107.7300000007</v>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>13774.47300000003</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>19489.66</v>
-      </c>
-      <c r="E24" s="11" t="n">
-        <v>-6627.168509433931</v>
-      </c>
-      <c r="F24" s="11" t="n">
-        <v>-107.2425283018929</v>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>-2756.317999999999</v>
-      </c>
-      <c r="H24" s="11" t="n">
-        <v>-3377.460000000003</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>0.1908735019376091</v>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>主要是推广前利润下降</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>6.22-6.28</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="n">
-        <v>86704.38000000019</v>
-      </c>
-      <c r="C25" s="10" t="n">
-        <v>11721.55400000001</v>
-      </c>
-      <c r="D25" s="14" t="n">
-        <v>17051.12</v>
-      </c>
-      <c r="E25" s="11" t="n">
-        <v>-6338.785622641502</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <v>288.3828867924285</v>
-      </c>
-      <c r="G25" s="11" t="n">
-        <v>-2052.91900000002</v>
-      </c>
-      <c r="H25" s="11" t="n">
-        <v>-2438.539999999997</v>
-      </c>
-      <c r="I25" s="15" t="n">
-        <v>0.1966581157722362</v>
-      </c>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>本期改善</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>6.29-7.5</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n">
-        <v>93257.14000000031</v>
-      </c>
-      <c r="C26" s="10" t="n">
-        <v>12985.26300000003</v>
-      </c>
-      <c r="D26" s="9" t="n">
-        <v>17356.51</v>
-      </c>
-      <c r="E26" s="11" t="n">
-        <v>-5229.755867924498</v>
-      </c>
-      <c r="F26" s="10" t="n">
-        <v>1109.029754717005</v>
-      </c>
-      <c r="G26" s="10" t="n">
-        <v>1263.709000000019</v>
-      </c>
-      <c r="H26" s="10" t="n">
-        <v>305.3899999999994</v>
-      </c>
-      <c r="I26" s="12" t="n">
-        <v>0.186114543079489</v>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>本期改善</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>7.6-7.12</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="n">
-        <v>120624.1200000009</v>
-      </c>
-      <c r="C27" s="10" t="n">
-        <v>16853.98700000001</v>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>20166.80900000001</v>
-      </c>
-      <c r="E27" s="11" t="n">
-        <v>-4108.993188679236</v>
-      </c>
-      <c r="F27" s="10" t="n">
-        <v>1120.762679245261</v>
-      </c>
-      <c r="G27" s="10" t="n">
-        <v>3868.723999999982</v>
-      </c>
-      <c r="H27" s="10" t="n">
-        <v>2810.299000000014</v>
-      </c>
-      <c r="I27" s="15" t="n">
-        <v>0.1671872010340872</v>
-      </c>
-      <c r="J27" s="13" t="inlineStr">
-        <is>
-          <t>本期改善</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>7.13-7.19</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="n">
-        <v>100698.0300000007</v>
-      </c>
-      <c r="C28" s="10" t="n">
-        <v>13663.37600000004</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <v>17570.48999999999</v>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>-5181.567396226362</v>
-      </c>
-      <c r="F28" s="11" t="n">
-        <v>-1072.574207547125</v>
-      </c>
-      <c r="G28" s="11" t="n">
-        <v>-3190.610999999972</v>
-      </c>
-      <c r="H28" s="11" t="n">
-        <v>-2596.319000000025</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>0.1744869288902659</v>
-      </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>主要是推广前利润下降</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>7.20-7.26</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
-        <v>98448.25000000061</v>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>13513.29000000004</v>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>18177.49</v>
-      </c>
-      <c r="E29" s="11" t="n">
-        <v>-5613.776037735816</v>
-      </c>
-      <c r="F29" s="11" t="n">
-        <v>-432.2086415094545</v>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>-150.0859999999975</v>
-      </c>
-      <c r="H29" s="10" t="n">
-        <v>607.0000000000146</v>
-      </c>
-      <c r="I29" s="15" t="n">
-        <v>0.1846400520070178</v>
-      </c>
-      <c r="J29" s="13" t="inlineStr">
-        <is>
-          <t>主要是推广费上升</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>7.27-8.2</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="n">
-        <v>107467.6600000008</v>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>15014.01200000004</v>
-      </c>
-      <c r="D30" s="9" t="n">
-        <v>19204.37726581657</v>
-      </c>
-      <c r="E30" s="11" t="n">
-        <v>-5109.368381499395</v>
-      </c>
-      <c r="F30" s="10" t="n">
-        <v>504.4076562364216</v>
-      </c>
-      <c r="G30" s="10" t="n">
-        <v>1500.722</v>
-      </c>
-      <c r="H30" s="10" t="n">
-        <v>1026.887265816571</v>
-      </c>
-      <c r="I30" s="12" t="n">
-        <v>0.1786991292619233</v>
-      </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>本期改善</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
           <t>ID周损益合计趋势（正确单周，已拆分7.20/7.27）</t>
         </is>
       </c>
@@ -1471,7 +1578,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2222,7 +2329,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2714,7 +2821,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3593,7 +3700,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -5196,7 +5303,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M91"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -8392,7 +8499,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -9146,7 +9253,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>

</xml_diff>